<commit_message>
n8n board refresh 2026-10-04T17:40:21Z
</commit_message>
<xml_diff>
--- a/app/reports/MPB_research.xlsx
+++ b/app/reports/MPB_research.xlsx
@@ -621,7 +621,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generated 2026-10-03 17:35 · Source: FMP · Methodology: financial-analysis plugin (Anthropic FSI), adapted for free-tier data</t>
+          <t>Generated 2026-10-04 17:35 · Source: FMP · Methodology: financial-analysis plugin (Anthropic FSI), adapted for free-tier data</t>
         </is>
       </c>
     </row>
@@ -1567,7 +1567,7 @@
         <v>849846272</v>
       </c>
       <c r="D7" s="34" t="n">
-        <v>13.568306</v>
+        <v>13.794445</v>
       </c>
       <c r="E7" s="34" t="n"/>
       <c r="F7" s="34" t="n">

</xml_diff>